<commit_message>
docs(QA-5687): evidencias E2E PASS — acuse 89728, rechazo 89729
Co-authored-by: JFCandia-Digital <JFCandia-Digital@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/api-v3.5/matriz_api_test_recepcion_integracion_DocDigital.xlsx
+++ b/docs/api-v3.5/matriz_api_test_recepcion_integracion_DocDigital.xlsx
@@ -609,7 +609,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -1617,7 +1617,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>24-06-2026</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">

</xml_diff>